<commit_message>
Analysing HFR TDI cases for calibration of ShearQ app, cases uploaded to FTP server. README file updated.
</commit_message>
<xml_diff>
--- a/data/raw/2026-09-13_hfr_tdi_calibration-cases_derived-from-SAS-F-5.xlsx
+++ b/data/raw/2026-09-13_hfr_tdi_calibration-cases_derived-from-SAS-F-5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studntnu-my.sharepoint.com/personal/kjellhoy_ntnu_no/Documents/Documents/PhD/05_Analyse-i-R/Sharing-of-data-in-PhD-project/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2346" documentId="11_AD4DB114E441178AC67DF4C8DE97C310693EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D974057C-EB93-45C0-8B69-D24085C43EEE}"/>
+  <xr:revisionPtr revIDLastSave="2456" documentId="11_AD4DB114E441178AC67DF4C8DE97C310693EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16F5FDDB-716D-47C6-8B21-23CA37B2E37D}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5460" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HFR TDI calibration cases" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="23">
   <si>
     <t>id</t>
   </si>
@@ -622,7 +622,7 @@
   <sheetPr>
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
-  <dimension ref="A1:P174"/>
+  <dimension ref="A1:P181"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="8"/>
@@ -8335,27 +8335,398 @@
       </c>
     </row>
     <row r="170" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A170" s="7">
+      <c r="A170" s="14">
         <v>62875</v>
+      </c>
+      <c r="B170" s="8">
+        <v>1</v>
+      </c>
+      <c r="C170" s="8">
+        <v>3</v>
+      </c>
+      <c r="D170" s="8">
+        <v>3</v>
+      </c>
+      <c r="E170" s="8">
+        <v>1</v>
+      </c>
+      <c r="F170" s="8">
+        <v>1</v>
+      </c>
+      <c r="G170" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="H170" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="I170" s="8">
+        <v>0.41</v>
+      </c>
+      <c r="J170" s="8">
+        <v>4</v>
+      </c>
+      <c r="K170" s="8">
+        <v>3</v>
+      </c>
+      <c r="L170" s="8">
+        <v>2</v>
+      </c>
+      <c r="M170" s="8">
+        <v>2</v>
+      </c>
+      <c r="N170" s="8">
+        <v>8</v>
+      </c>
+      <c r="O170" s="8" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="171" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A171" s="7">
-        <v>66497</v>
+        <v>62875</v>
+      </c>
+      <c r="B171" s="8">
+        <v>1</v>
+      </c>
+      <c r="C171" s="8">
+        <v>3</v>
+      </c>
+      <c r="D171" s="8">
+        <v>3</v>
+      </c>
+      <c r="E171" s="8">
+        <v>2</v>
+      </c>
+      <c r="F171" s="8">
+        <v>2</v>
+      </c>
+      <c r="G171" s="8">
+        <v>5.5</v>
+      </c>
+      <c r="H171" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="I171" s="8">
+        <v>0.64</v>
+      </c>
+      <c r="J171" s="8">
+        <v>4</v>
+      </c>
+      <c r="K171" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="L171" s="8">
+        <v>2</v>
+      </c>
+      <c r="M171" s="8">
+        <v>2</v>
+      </c>
+      <c r="N171" s="8">
+        <v>8</v>
+      </c>
+      <c r="O171" s="8" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="172" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A172" s="7">
-        <v>77614</v>
+        <v>62875</v>
+      </c>
+      <c r="B172" s="8">
+        <v>1</v>
+      </c>
+      <c r="C172" s="8">
+        <v>3</v>
+      </c>
+      <c r="D172" s="8">
+        <v>3</v>
+      </c>
+      <c r="E172" s="8">
+        <v>3</v>
+      </c>
+      <c r="F172" s="8">
+        <v>3</v>
+      </c>
+      <c r="G172" s="8">
+        <v>5.7</v>
+      </c>
+      <c r="H172" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I172" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J172" s="8">
+        <v>5</v>
+      </c>
+      <c r="K172" s="8">
+        <v>2.75</v>
+      </c>
+      <c r="L172" s="8">
+        <v>2</v>
+      </c>
+      <c r="M172" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="N172" s="8">
+        <v>8</v>
+      </c>
+      <c r="O172" s="8" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="173" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A173" s="7">
-        <v>83354</v>
+        <v>62875</v>
+      </c>
+      <c r="B173" s="8">
+        <v>1</v>
+      </c>
+      <c r="C173" s="8">
+        <v>3</v>
+      </c>
+      <c r="D173" s="8">
+        <v>3</v>
+      </c>
+      <c r="E173" s="8">
+        <v>4</v>
+      </c>
+      <c r="F173" s="8">
+        <v>4</v>
+      </c>
+      <c r="G173" s="8">
+        <v>6.5</v>
+      </c>
+      <c r="H173" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I173" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J173" s="8">
+        <v>4</v>
+      </c>
+      <c r="K173" s="8">
+        <v>2.25</v>
+      </c>
+      <c r="L173" s="8">
+        <v>2</v>
+      </c>
+      <c r="M173" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="N173" s="8">
+        <v>8</v>
+      </c>
+      <c r="O173" s="8" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="174" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A174" s="7">
+        <v>62875</v>
+      </c>
+      <c r="B174" s="8">
+        <v>2</v>
+      </c>
+      <c r="C174" s="8">
+        <v>3</v>
+      </c>
+      <c r="D174" s="8">
+        <v>3</v>
+      </c>
+      <c r="E174" s="8">
+        <v>5</v>
+      </c>
+      <c r="F174" s="8">
+        <v>1</v>
+      </c>
+      <c r="G174" s="8">
+        <v>9</v>
+      </c>
+      <c r="H174" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I174" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J174" s="8">
+        <v>4</v>
+      </c>
+      <c r="K174" s="8">
+        <v>3</v>
+      </c>
+      <c r="L174" s="8">
+        <v>3</v>
+      </c>
+      <c r="M174" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="N174" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="O174" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="175" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A175" s="7">
+        <v>62875</v>
+      </c>
+      <c r="B175" s="8">
+        <v>2</v>
+      </c>
+      <c r="C175" s="8">
+        <v>3</v>
+      </c>
+      <c r="D175" s="8">
+        <v>3</v>
+      </c>
+      <c r="E175" s="8">
+        <v>6</v>
+      </c>
+      <c r="F175" s="8">
+        <v>2</v>
+      </c>
+      <c r="G175" s="8">
+        <v>8.6</v>
+      </c>
+      <c r="H175" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I175" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J175" s="8">
+        <v>4</v>
+      </c>
+      <c r="K175" s="8">
+        <v>2.75</v>
+      </c>
+      <c r="L175" s="8">
+        <v>3</v>
+      </c>
+      <c r="M175" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="N175" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="O175" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="176" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A176" s="7">
+        <v>62875</v>
+      </c>
+      <c r="B176" s="8">
+        <v>2</v>
+      </c>
+      <c r="C176" s="8">
+        <v>3</v>
+      </c>
+      <c r="D176" s="8">
+        <v>3</v>
+      </c>
+      <c r="E176" s="8">
+        <v>7</v>
+      </c>
+      <c r="F176" s="8">
+        <v>3</v>
+      </c>
+      <c r="G176" s="8">
+        <v>5.5</v>
+      </c>
+      <c r="H176" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="I176" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="J176" s="8">
+        <v>5</v>
+      </c>
+      <c r="K176" s="8">
+        <v>3</v>
+      </c>
+      <c r="L176" s="8">
+        <v>2</v>
+      </c>
+      <c r="M176" s="8">
+        <v>2</v>
+      </c>
+      <c r="N176" s="8">
+        <v>8</v>
+      </c>
+      <c r="O176" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="177" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A177" s="7">
+        <v>62875</v>
+      </c>
+      <c r="B177" s="8">
+        <v>2</v>
+      </c>
+      <c r="C177" s="8">
+        <v>3</v>
+      </c>
+      <c r="D177" s="8">
+        <v>3</v>
+      </c>
+      <c r="E177" s="8">
+        <v>8</v>
+      </c>
+      <c r="F177" s="8">
+        <v>4</v>
+      </c>
+      <c r="G177" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="H177" s="8">
+        <v>5.8</v>
+      </c>
+      <c r="I177" s="8">
+        <v>0.39</v>
+      </c>
+      <c r="J177" s="8">
+        <v>4</v>
+      </c>
+      <c r="K177" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="L177" s="8">
+        <v>2</v>
+      </c>
+      <c r="M177" s="8">
+        <v>2</v>
+      </c>
+      <c r="N177" s="8">
+        <v>8</v>
+      </c>
+      <c r="O177" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="178" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A178" s="14">
+        <v>66497</v>
+      </c>
+    </row>
+    <row r="179" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A179" s="7">
+        <v>77614</v>
+      </c>
+    </row>
+    <row r="180" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A180" s="7">
+        <v>83354</v>
+      </c>
+    </row>
+    <row r="181" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A181" s="7">
         <v>92849</v>
       </c>
     </row>
@@ -8781,7 +9152,7 @@
         <v>2</v>
       </c>
       <c r="E21" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" s="19">
         <v>0</v>

</xml_diff>